<commit_message>
fix output + result update
</commit_message>
<xml_diff>
--- a/results/2026-04-07-SAT-precedence-graph/Tóm tắt kết quả.xlsx
+++ b/results/2026-04-07-SAT-precedence-graph/Tóm tắt kết quả.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\maxsattrainscheduling\results\2026-04-04-SAT-initial-synchronous-heuristic\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\maxsattrainscheduling\results\2026-04-07-SAT-precedence-graph\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1204,67 +1204,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="60" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="64" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="38" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="39" xfId="2" applyBorder="1"/>
@@ -1317,6 +1260,63 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="73" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="75" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent2" xfId="2" builtinId="34"/>
@@ -1642,195 +1642,219 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="61" t="s">
+      <c r="A1" s="101" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="104" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="75" t="s">
+      <c r="C1" s="112" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
-      <c r="P1" s="78"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+      <c r="H1" s="113"/>
+      <c r="I1" s="113"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="113"/>
+      <c r="L1" s="113"/>
+      <c r="M1" s="113"/>
+      <c r="N1" s="113"/>
+      <c r="O1" s="113"/>
+      <c r="P1" s="113"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="68"/>
-      <c r="B2" s="69"/>
-      <c r="C2" s="76" t="s">
+      <c r="A2" s="102"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="116" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-      <c r="K2" s="77" t="s">
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="77"/>
-      <c r="M2" s="77"/>
-      <c r="N2" s="77"/>
-      <c r="O2" s="77"/>
-      <c r="P2" s="77"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
     </row>
     <row r="3" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="60"/>
-      <c r="B3" s="62"/>
-      <c r="C3" s="64" t="s">
+      <c r="A3" s="103"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="71"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="66" t="s">
+      <c r="D3" s="115"/>
+      <c r="E3" s="109"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="71"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="64" t="s">
+      <c r="H3" s="115"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="110"/>
+      <c r="K3" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="65"/>
-      <c r="M3" s="65"/>
-      <c r="N3" s="66" t="s">
+      <c r="L3" s="109"/>
+      <c r="M3" s="109"/>
+      <c r="N3" s="108" t="s">
         <v>4</v>
       </c>
-      <c r="O3" s="65"/>
-      <c r="P3" s="67"/>
+      <c r="O3" s="109"/>
+      <c r="P3" s="110"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="60"/>
-      <c r="B4" s="63"/>
-      <c r="C4" s="96" t="s">
+      <c r="A4" s="103"/>
+      <c r="B4" s="107"/>
+      <c r="C4" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="97" t="s">
+      <c r="D4" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="98" t="s">
+      <c r="E4" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="99" t="s">
+      <c r="F4" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="100" t="s">
+      <c r="G4" s="81" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="98" t="s">
+      <c r="H4" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="101" t="s">
+      <c r="I4" s="82" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="102" t="s">
+      <c r="J4" s="83" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="96" t="s">
+      <c r="K4" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="98" t="s">
+      <c r="L4" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="99" t="s">
+      <c r="M4" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="100" t="s">
+      <c r="N4" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="101" t="s">
+      <c r="O4" s="82" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="102" t="s">
+      <c r="P4" s="83" t="s">
         <v>14</v>
       </c>
       <c r="Q4" s="53"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="56" t="s">
+      <c r="A5" s="98" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="103">
+      <c r="C5" s="84">
         <v>11763.28</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="3"/>
       <c r="F5" s="4"/>
-      <c r="G5" s="116"/>
+      <c r="G5" s="97"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="3"/>
+      <c r="K5" s="2">
+        <v>41110.400000000001</v>
+      </c>
+      <c r="L5" s="3">
+        <v>17211.82</v>
+      </c>
       <c r="M5" s="4"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="6"/>
+      <c r="N5" s="5">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6">
+        <v>21</v>
+      </c>
       <c r="P5" s="7"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="56"/>
+      <c r="A6" s="98"/>
       <c r="B6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="104">
+      <c r="C6" s="85">
         <v>23035.61</v>
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="10"/>
       <c r="F6" s="11"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="72"/>
+      <c r="H6" s="57"/>
       <c r="I6" s="10"/>
       <c r="J6" s="54"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="10"/>
+      <c r="K6" s="9">
+        <v>53576.2</v>
+      </c>
+      <c r="L6" s="10">
+        <v>22764.01</v>
+      </c>
       <c r="M6" s="11"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="10"/>
+      <c r="N6" s="12">
+        <v>14</v>
+      </c>
+      <c r="O6" s="10">
+        <v>20</v>
+      </c>
       <c r="P6" s="54"/>
       <c r="Q6" s="53"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56"/>
+      <c r="A7" s="98"/>
       <c r="B7" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="105">
+      <c r="C7" s="86">
         <v>42557.14</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
       <c r="F7" s="16"/>
-      <c r="G7" s="113"/>
-      <c r="H7" s="107"/>
+      <c r="G7" s="94"/>
+      <c r="H7" s="88"/>
       <c r="I7" s="15"/>
       <c r="J7" s="55"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="15"/>
+      <c r="K7" s="14">
+        <v>60763.3</v>
+      </c>
+      <c r="L7" s="15">
+        <v>42734.62</v>
+      </c>
       <c r="M7" s="16"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="15"/>
+      <c r="N7" s="17">
+        <v>14</v>
+      </c>
+      <c r="O7" s="15">
+        <v>16</v>
+      </c>
       <c r="P7" s="55"/>
     </row>
     <row r="8" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56"/>
+      <c r="A8" s="98"/>
       <c r="B8" s="22" t="s">
         <v>10</v>
       </c>
@@ -1838,7 +1862,7 @@
         <f>SUM(C5:C7)</f>
         <v>77356.03</v>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="58">
         <f>SUM(D5:D7)</f>
         <v>0</v>
       </c>
@@ -1850,11 +1874,11 @@
         <f t="shared" ref="F8:J8" si="0">SUM(F5:F7)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="114">
+      <c r="G8" s="95">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="115">
+      <c r="H8" s="96">
         <f t="shared" ref="H8" si="1">SUM(H5:H7)</f>
         <v>0</v>
       </c>
@@ -1866,34 +1890,34 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K8" s="79">
+      <c r="K8" s="60">
         <f>SUM(K5:K7)</f>
-        <v>0</v>
-      </c>
-      <c r="L8" s="80">
+        <v>155449.90000000002</v>
+      </c>
+      <c r="L8" s="61">
         <f>SUM(L5:L7)</f>
-        <v>0</v>
-      </c>
-      <c r="M8" s="81">
+        <v>82710.450000000012</v>
+      </c>
+      <c r="M8" s="62">
         <f t="shared" ref="M8:N8" si="2">SUM(M5:M7)</f>
         <v>0</v>
       </c>
-      <c r="N8" s="82">
+      <c r="N8" s="63">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O8" s="83">
+        <v>44</v>
+      </c>
+      <c r="O8" s="64">
         <f t="shared" ref="O8:P8" si="3">SUM(O5:O7)</f>
-        <v>0</v>
-      </c>
-      <c r="P8" s="81">
+        <v>57</v>
+      </c>
+      <c r="P8" s="62">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q8" s="53"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="99" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="27" t="s">
@@ -1905,19 +1929,27 @@
       <c r="D9" s="28"/>
       <c r="E9" s="29"/>
       <c r="F9" s="30"/>
-      <c r="G9" s="111"/>
-      <c r="H9" s="95"/>
+      <c r="G9" s="92"/>
+      <c r="H9" s="76"/>
       <c r="I9" s="3"/>
       <c r="J9" s="32"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="29"/>
+      <c r="K9" s="28">
+        <v>26.39076</v>
+      </c>
+      <c r="L9" s="29">
+        <v>58.932989999999997</v>
+      </c>
       <c r="M9" s="30"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="3"/>
+      <c r="N9" s="31">
+        <v>24</v>
+      </c>
+      <c r="O9" s="3">
+        <v>24</v>
+      </c>
       <c r="P9" s="32"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="57"/>
+      <c r="A10" s="99"/>
       <c r="B10" s="33" t="s">
         <v>8</v>
       </c>
@@ -1928,19 +1960,27 @@
       <c r="E10" s="34"/>
       <c r="F10" s="11"/>
       <c r="G10" s="35"/>
-      <c r="H10" s="74"/>
+      <c r="H10" s="59"/>
       <c r="I10" s="34"/>
-      <c r="J10" s="92"/>
-      <c r="K10" s="74"/>
-      <c r="L10" s="34"/>
+      <c r="J10" s="73"/>
+      <c r="K10" s="59">
+        <v>15319.75</v>
+      </c>
+      <c r="L10" s="34">
+        <v>10019.17</v>
+      </c>
       <c r="M10" s="11"/>
-      <c r="N10" s="35"/>
-      <c r="O10" s="34"/>
+      <c r="N10" s="35">
+        <v>21</v>
+      </c>
+      <c r="O10" s="34">
+        <v>23</v>
+      </c>
       <c r="P10" s="54"/>
       <c r="Q10" s="53"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="57"/>
+      <c r="A11" s="99"/>
       <c r="B11" s="36" t="s">
         <v>9</v>
       </c>
@@ -1950,23 +1990,31 @@
       <c r="D11" s="20"/>
       <c r="E11" s="37"/>
       <c r="F11" s="21"/>
-      <c r="G11" s="109"/>
+      <c r="G11" s="90"/>
       <c r="H11" s="15"/>
       <c r="I11" s="37"/>
       <c r="J11" s="18"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="37"/>
+      <c r="K11" s="20">
+        <v>15894.96</v>
+      </c>
+      <c r="L11" s="37">
+        <v>835.88440000000003</v>
+      </c>
       <c r="M11" s="21"/>
-      <c r="N11" s="38"/>
-      <c r="O11" s="37"/>
+      <c r="N11" s="38">
+        <v>21</v>
+      </c>
+      <c r="O11" s="37">
+        <v>24</v>
+      </c>
       <c r="P11" s="18"/>
     </row>
     <row r="12" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="57"/>
+      <c r="A12" s="99"/>
       <c r="B12" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="70">
+      <c r="C12" s="56">
         <f>SUM(C9:C11)</f>
         <v>22272.202149999997</v>
       </c>
@@ -1982,7 +2030,7 @@
         <f t="shared" ref="F12:I12" si="4">SUM(F9:F11)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="112">
+      <c r="G12" s="93">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -1998,33 +2046,33 @@
         <f>SUM(J9:J11)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="79">
+      <c r="K12" s="60">
         <f>SUM(K9:K11)</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="83">
+        <v>31241.100760000001</v>
+      </c>
+      <c r="L12" s="64">
         <f>SUM(L9:L11)</f>
-        <v>0</v>
-      </c>
-      <c r="M12" s="84">
-        <f t="shared" ref="M12:N12" si="6">SUM(M9:M11)</f>
-        <v>0</v>
-      </c>
-      <c r="N12" s="82">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="O12" s="83">
-        <f t="shared" ref="O12:P12" si="7">SUM(O9:O11)</f>
-        <v>0</v>
-      </c>
-      <c r="P12" s="85">
+        <v>10913.98739</v>
+      </c>
+      <c r="M12" s="65">
+        <f t="shared" ref="M12" si="6">SUM(M9:M11)</f>
+        <v>0</v>
+      </c>
+      <c r="N12" s="63">
+        <f>SUM(N9:N11)</f>
+        <v>66</v>
+      </c>
+      <c r="O12" s="64">
+        <f t="shared" ref="O12" si="7">SUM(O9:O11)</f>
+        <v>71</v>
+      </c>
+      <c r="P12" s="66">
         <f>SUM(P9:P11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" s="56" t="s">
+      <c r="A13" s="98" t="s">
         <v>12</v>
       </c>
       <c r="B13" s="43" t="s">
@@ -2036,74 +2084,98 @@
       <c r="D13" s="44"/>
       <c r="E13" s="3"/>
       <c r="F13" s="45"/>
-      <c r="G13" s="111"/>
-      <c r="H13" s="95"/>
+      <c r="G13" s="92"/>
+      <c r="H13" s="76"/>
       <c r="I13" s="3"/>
       <c r="J13" s="45"/>
-      <c r="K13" s="93"/>
-      <c r="L13" s="3"/>
+      <c r="K13" s="74">
+        <v>43.055619999999998</v>
+      </c>
+      <c r="L13" s="3">
+        <v>45.864530000000002</v>
+      </c>
       <c r="M13" s="45"/>
-      <c r="N13" s="31"/>
-      <c r="O13" s="3"/>
+      <c r="N13" s="31">
+        <v>24</v>
+      </c>
+      <c r="O13" s="3">
+        <v>24</v>
+      </c>
       <c r="P13" s="45"/>
       <c r="Q13" s="53"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" s="56"/>
+      <c r="A14" s="98"/>
       <c r="B14" s="46" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="9">
         <v>24.887712709999999</v>
       </c>
-      <c r="D14" s="72"/>
+      <c r="D14" s="57"/>
       <c r="E14" s="10"/>
       <c r="F14" s="11"/>
-      <c r="G14" s="110"/>
+      <c r="G14" s="91"/>
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
       <c r="J14" s="11"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="10"/>
+      <c r="K14" s="9">
+        <v>5177.1679999999997</v>
+      </c>
+      <c r="L14" s="10">
+        <v>38.798310000000001</v>
+      </c>
       <c r="M14" s="11"/>
-      <c r="N14" s="35"/>
-      <c r="O14" s="10"/>
+      <c r="N14" s="35">
+        <v>23</v>
+      </c>
+      <c r="O14" s="10">
+        <v>24</v>
+      </c>
       <c r="P14" s="11"/>
       <c r="Q14" s="53"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="56"/>
+      <c r="A15" s="98"/>
       <c r="B15" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="106">
+      <c r="C15" s="87">
         <v>26.39</v>
       </c>
-      <c r="D15" s="107"/>
+      <c r="D15" s="88"/>
       <c r="E15" s="20"/>
       <c r="F15" s="21"/>
-      <c r="G15" s="109"/>
+      <c r="G15" s="90"/>
       <c r="H15" s="15"/>
       <c r="I15" s="20"/>
       <c r="J15" s="21"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="20"/>
+      <c r="K15" s="19">
+        <v>328.22469999999998</v>
+      </c>
+      <c r="L15" s="20">
+        <v>72.841210000000004</v>
+      </c>
       <c r="M15" s="21"/>
-      <c r="N15" s="38"/>
-      <c r="O15" s="20"/>
+      <c r="N15" s="38">
+        <v>24</v>
+      </c>
+      <c r="O15" s="20">
+        <v>24</v>
+      </c>
       <c r="P15" s="21"/>
       <c r="Q15" s="53"/>
     </row>
     <row r="16" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="58"/>
+      <c r="A16" s="100"/>
       <c r="B16" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="108">
+      <c r="C16" s="89">
         <f>SUM(C13:C15)</f>
         <v>57.597884839999999</v>
       </c>
-      <c r="D16" s="94">
+      <c r="D16" s="75">
         <f>SUM(D13:D15)</f>
         <v>0</v>
       </c>
@@ -2131,33 +2203,33 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="K16" s="86">
+      <c r="K16" s="67">
         <f>SUM(K13:K15)</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="87">
+        <v>5548.4483199999995</v>
+      </c>
+      <c r="L16" s="68">
         <f>SUM(L13:L15)</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="88">
-        <f t="shared" ref="M16:N16" si="10">SUM(M13:M15)</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="89">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="87">
+        <v>157.50405000000001</v>
+      </c>
+      <c r="M16" s="69">
+        <f t="shared" ref="M16" si="10">SUM(M13:M15)</f>
+        <v>0</v>
+      </c>
+      <c r="N16" s="70">
+        <f>SUM(N13:N15)</f>
+        <v>71</v>
+      </c>
+      <c r="O16" s="68">
         <f t="shared" ref="O16:P16" si="11">SUM(O13:O15)</f>
-        <v>0</v>
-      </c>
-      <c r="P16" s="90">
+        <v>72</v>
+      </c>
+      <c r="P16" s="71">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="4:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="91"/>
+      <c r="D17" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>